<commit_message>
update dataloader for ALL stage
</commit_message>
<xml_diff>
--- a/notes.xlsx
+++ b/notes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deveshshah/Documents/Programming/Out_Of_Distribution_Exploration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A750DB9A-ADC0-AD46-9029-E098952A96E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE391562-09B9-624A-8473-F1334381813E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="920" windowWidth="14900" windowHeight="16860" activeTab="1" xr2:uid="{7A4485C0-0849-FB48-8E6E-A312C4571800}"/>
+    <workbookView xWindow="220" yWindow="840" windowWidth="15640" windowHeight="16860" xr2:uid="{7A4485C0-0849-FB48-8E6E-A312C4571800}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="59">
   <si>
     <t>Datasets</t>
   </si>
@@ -211,13 +211,16 @@
   </si>
   <si>
     <t>1184 (8%)</t>
+  </si>
+  <si>
+    <t>normal 5-class with BCE loss</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -230,6 +233,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -250,10 +261,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -268,8 +280,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -602,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD9FA183-F003-A644-A137-AE4E9F460B97}">
-  <dimension ref="A2:F30"/>
+  <dimension ref="A2:F31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="6" width="24.5" customWidth="1"/>
@@ -648,7 +662,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="F5" t="s">
@@ -728,7 +742,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -736,51 +750,45 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
         <v>17</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C25" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D25" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D26" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>4</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>5</v>
+      </c>
+      <c r="B28" t="s">
         <v>18</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>20</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D28" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D28" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D29" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29">
-        <v>5</v>
-      </c>
-      <c r="B29" t="s">
-        <v>19</v>
-      </c>
-      <c r="C29" t="s">
-        <v>21</v>
-      </c>
-      <c r="D29" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -788,16 +796,34 @@
         <v>6</v>
       </c>
       <c r="B30" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>7</v>
+      </c>
+      <c r="B31" t="s">
         <v>23</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>24</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D31" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{B7D0DF65-64A0-C244-A280-92BC7FF1B7BA}"/>
+    <hyperlink ref="C25" r:id="rId2" xr:uid="{48781F69-BFC8-AD40-9498-4047C51304E6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>